<commit_message>
Cleaned up repo by adding an archive folder + fixed constant coolant mass flow error in main
</commit_message>
<xml_diff>
--- a/REGEN/Contour_Maelstrom.xlsx
+++ b/REGEN/Contour_Maelstrom.xlsx
@@ -85,7 +85,7 @@
     </row>
     <row r="3">
       <c r="A3" s="0">
-        <v>0.00062749449081803002</v>
+        <v>0.00062749449081803003</v>
       </c>
       <c r="B3" s="0">
         <v>0.042227500000000001</v>
@@ -272,7 +272,7 @@
     </row>
     <row r="20">
       <c r="A20" s="0">
-        <v>0.0059611976627712854</v>
+        <v>0.0059611976627712855</v>
       </c>
       <c r="B20" s="0">
         <v>0.042227500000000001</v>
@@ -778,7 +778,7 @@
     </row>
     <row r="66">
       <c r="A66" s="0">
-        <v>0.020393570951585976</v>
+        <v>0.020393570951585977</v>
       </c>
       <c r="B66" s="0">
         <v>0.042227500000000001</v>
@@ -844,7 +844,7 @@
     </row>
     <row r="72">
       <c r="A72" s="0">
-        <v>0.022276054424040063</v>
+        <v>0.022276054424040064</v>
       </c>
       <c r="B72" s="0">
         <v>0.042227500000000001</v>
@@ -1141,7 +1141,7 @@
     </row>
     <row r="99">
       <c r="A99" s="0">
-        <v>0.030747230050083472</v>
+        <v>0.030747230050083473</v>
       </c>
       <c r="B99" s="0">
         <v>0.042227500000000001</v>
@@ -2109,7 +2109,7 @@
     </row>
     <row r="187">
       <c r="A187" s="0">
-        <v>0.058356987646076781</v>
+        <v>0.058356987646076782</v>
       </c>
       <c r="B187" s="0">
         <v>0.042227500000000001</v>
@@ -2538,7 +2538,7 @@
     </row>
     <row r="226">
       <c r="A226" s="0">
-        <v>0.070593130217028371</v>
+        <v>0.070593130217028372</v>
       </c>
       <c r="B226" s="0">
         <v>0.042227500000000001</v>
@@ -2571,7 +2571,7 @@
     </row>
     <row r="229">
       <c r="A229" s="0">
-        <v>0.071534371953255418</v>
+        <v>0.071534371953255419</v>
       </c>
       <c r="B229" s="0">
         <v>0.042227500000000001</v>
@@ -2703,7 +2703,7 @@
     </row>
     <row r="241">
       <c r="A241" s="0">
-        <v>0.075299338898163592</v>
+        <v>0.075299338898163593</v>
       </c>
       <c r="B241" s="0">
         <v>0.042227500000000001</v>
@@ -2736,7 +2736,7 @@
     </row>
     <row r="244">
       <c r="A244" s="0">
-        <v>0.076240580634390639</v>
+        <v>0.07624058063439064</v>
       </c>
       <c r="B244" s="0">
         <v>0.042227500000000001</v>
@@ -2769,7 +2769,7 @@
     </row>
     <row r="247">
       <c r="A247" s="0">
-        <v>0.077181822370617686</v>
+        <v>0.077181822370617687</v>
       </c>
       <c r="B247" s="0">
         <v>0.042227500000000001</v>
@@ -2802,7 +2802,7 @@
     </row>
     <row r="250">
       <c r="A250" s="0">
-        <v>0.078123064106844733</v>
+        <v>0.078123064106844734</v>
       </c>
       <c r="B250" s="0">
         <v>0.042227500000000001</v>
@@ -2835,7 +2835,7 @@
     </row>
     <row r="253">
       <c r="A253" s="0">
-        <v>0.07906430584307178</v>
+        <v>0.079064305843071781</v>
       </c>
       <c r="B253" s="0">
         <v>0.042227500000000001</v>
@@ -2868,7 +2868,7 @@
     </row>
     <row r="256">
       <c r="A256" s="0">
-        <v>0.080005547579298827</v>
+        <v>0.080005547579298828</v>
       </c>
       <c r="B256" s="0">
         <v>0.042227500000000001</v>
@@ -3512,7 +3512,7 @@
         <v>0.042203368288967008</v>
       </c>
       <c r="C314" s="0">
-        <v>6.3425806917742253</v>
+        <v>6.3425806917742254</v>
       </c>
     </row>
     <row r="315">
@@ -3520,7 +3520,7 @@
         <v>0.09851663505843071</v>
       </c>
       <c r="B315" s="0">
-        <v>0.042180095081803939</v>
+        <v>0.04218009508180394</v>
       </c>
       <c r="C315" s="0">
         <v>6.3355873403087175</v>
@@ -3531,7 +3531,7 @@
         <v>0.098830382303839726</v>
       </c>
       <c r="B316" s="0">
-        <v>0.042148982205388381</v>
+        <v>0.042148982205388382</v>
       </c>
       <c r="C316" s="0">
         <v>6.3262442771244309</v>
@@ -3567,7 +3567,7 @@
         <v>0.042007945397639204</v>
       </c>
       <c r="C319" s="0">
-        <v>6.2839779884431239</v>
+        <v>6.283977988443124</v>
       </c>
     </row>
     <row r="320">
@@ -3578,7 +3578,7 @@
         <v>0.041944732759688685</v>
       </c>
       <c r="C320" s="0">
-        <v>6.2650802321928047</v>
+        <v>6.2650802321928048</v>
       </c>
     </row>
     <row r="321">
@@ -3619,7 +3619,7 @@
         <v>0.10134036026711184</v>
       </c>
       <c r="B324" s="0">
-        <v>0.041607381252213554</v>
+        <v>0.041607381252213555</v>
       </c>
       <c r="C324" s="0">
         <v>6.1647083954616138</v>
@@ -3696,7 +3696,7 @@
         <v>0.10353659098497495</v>
       </c>
       <c r="B331" s="0">
-        <v>0.040657711779351353</v>
+        <v>0.040657711779351354</v>
       </c>
       <c r="C331" s="0">
         <v>5.8865066537798594</v>
@@ -3960,7 +3960,7 @@
         <v>0.11106652487479129</v>
       </c>
       <c r="B355" s="0">
-        <v>0.033841838842068261</v>
+        <v>0.033841838842068262</v>
       </c>
       <c r="C355" s="0">
         <v>4.0783047910023162</v>
@@ -3993,7 +3993,7 @@
         <v>0.11200776661101834</v>
       </c>
       <c r="B358" s="0">
-        <v>0.032900597105841214</v>
+        <v>0.032900597105841215</v>
       </c>
       <c r="C358" s="0">
         <v>3.8546001453147483</v>
@@ -4018,7 +4018,7 @@
         <v>0.032273102615023183</v>
       </c>
       <c r="C360" s="0">
-        <v>3.7089690667050021</v>
+        <v>3.7089690667050022</v>
       </c>
     </row>
     <row r="361">
@@ -4026,7 +4026,7 @@
         <v>0.11294900834724539</v>
       </c>
       <c r="B361" s="0">
-        <v>0.031959355369614167</v>
+        <v>0.031959355369614168</v>
       </c>
       <c r="C361" s="0">
         <v>3.6372051329547186</v>
@@ -4040,7 +4040,7 @@
         <v>0.031645608124205138</v>
       </c>
       <c r="C362" s="0">
-        <v>3.5661422695741591</v>
+        <v>3.5661422695741592</v>
       </c>
     </row>
     <row r="363">
@@ -4389,7 +4389,7 @@
         <v>0.12330266744574289</v>
       </c>
       <c r="B394" s="0">
-        <v>0.021605696271116664</v>
+        <v>0.021605696271116665</v>
       </c>
       <c r="C394" s="0">
         <v>1.6622957966119527</v>
@@ -4425,7 +4425,7 @@
         <v>0.020667852944765606</v>
       </c>
       <c r="C397" s="0">
-        <v>1.5211165766901273</v>
+        <v>1.5211165766901274</v>
       </c>
     </row>
     <row r="398">
@@ -4535,7 +4535,7 @@
         <v>0.018391478244757703</v>
       </c>
       <c r="C407" s="0">
-        <v>1.2044951318913903</v>
+        <v>1.2044951318913904</v>
       </c>
     </row>
     <row r="408">
@@ -4579,7 +4579,7 @@
         <v>0.017802430869026852</v>
       </c>
       <c r="C411" s="0">
-        <v>1.1285749061820975</v>
+        <v>1.1285749061820976</v>
       </c>
     </row>
     <row r="412">
@@ -4752,7 +4752,7 @@
         <v>0.13365632654424037</v>
       </c>
       <c r="B427" s="0">
-        <v>0.016760475384550329</v>
+        <v>0.01676047538455033</v>
       </c>
       <c r="C427" s="0">
         <v>1.0003326376227799</v>
@@ -4851,7 +4851,7 @@
         <v>0.13648005175292152</v>
       </c>
       <c r="B436" s="0">
-        <v>0.016991012948391004</v>
+        <v>0.016991012948391005</v>
       </c>
       <c r="C436" s="0">
         <v>1.0280407156322902</v>
@@ -4876,7 +4876,7 @@
         <v>0.017122125604231205</v>
       </c>
       <c r="C438" s="0">
-        <v>1.04396786549075</v>
+        <v>1.0439678654907501</v>
       </c>
     </row>
     <row r="439">
@@ -5159,7 +5159,7 @@
         <v>0.14526497462437393</v>
       </c>
       <c r="B464" s="0">
-        <v>0.01908022928940627</v>
+        <v>0.019080229289406271</v>
       </c>
       <c r="C464" s="0">
         <v>1.2963997908657239</v>
@@ -5170,7 +5170,7 @@
         <v>0.14557872186978296</v>
       </c>
       <c r="B465" s="0">
-        <v>0.019155553338748878</v>
+        <v>0.019155553338748879</v>
       </c>
       <c r="C465" s="0">
         <v>1.306655729573365</v>
@@ -5211,7 +5211,7 @@
     </row>
     <row r="469">
       <c r="A469" s="0">
-        <v>0.14683371085141902</v>
+        <v>0.14683371085141903</v>
       </c>
       <c r="B469" s="0">
         <v>0.019456849536119283</v>
@@ -5250,7 +5250,7 @@
         <v>0.019682821684147079</v>
       </c>
       <c r="C472" s="0">
-        <v>1.3795787290393386</v>
+        <v>1.3795787290393387</v>
       </c>
     </row>
     <row r="473">
@@ -5335,7 +5335,7 @@
         <v>0.15028493055091818</v>
       </c>
       <c r="B480" s="0">
-        <v>0.020285414078887887</v>
+        <v>0.020285414078887888</v>
       </c>
       <c r="C480" s="0">
         <v>1.4653437895272288</v>
@@ -5343,10 +5343,10 @@
     </row>
     <row r="481">
       <c r="A481" s="0">
-        <v>0.15059867779632718</v>
+        <v>0.15059867779632719</v>
       </c>
       <c r="B481" s="0">
-        <v>0.020360738128230488</v>
+        <v>0.020360738128230489</v>
       </c>
       <c r="C481" s="0">
         <v>1.4762462588134375</v>
@@ -5354,7 +5354,7 @@
     </row>
     <row r="482">
       <c r="A482" s="0">
-        <v>0.15091242504173621</v>
+        <v>0.15091242504173622</v>
       </c>
       <c r="B482" s="0">
         <v>0.02043606217757309</v>
@@ -5365,7 +5365,7 @@
     </row>
     <row r="483">
       <c r="A483" s="0">
-        <v>0.15122617228714524</v>
+        <v>0.15122617228714525</v>
       </c>
       <c r="B483" s="0">
         <v>0.020511386226915698</v>
@@ -5437,7 +5437,7 @@
         <v>0.020963330522971297</v>
       </c>
       <c r="C489" s="0">
-        <v>1.564920706904886</v>
+        <v>1.5649207069048861</v>
       </c>
     </row>
     <row r="490">
@@ -5486,7 +5486,7 @@
     </row>
     <row r="494">
       <c r="A494" s="0">
-        <v>0.15467739198664437</v>
+        <v>0.15467739198664438</v>
       </c>
       <c r="B494" s="0">
         <v>0.021339950769684295</v>
@@ -5497,7 +5497,7 @@
     </row>
     <row r="495">
       <c r="A495" s="0">
-        <v>0.1549911392320534</v>
+        <v>0.15499113923205341</v>
       </c>
       <c r="B495" s="0">
         <v>0.021415274819026903</v>
@@ -5522,7 +5522,7 @@
         <v>0.15561863372287144</v>
       </c>
       <c r="B497" s="0">
-        <v>0.021565922917712105</v>
+        <v>0.021565922917712106</v>
       </c>
       <c r="C497" s="0">
         <v>1.6561812773106099</v>
@@ -5580,7 +5580,7 @@
         <v>0.021942543164425104</v>
       </c>
       <c r="C502" s="0">
-        <v>1.7145323990519032</v>
+        <v>1.7145323990519033</v>
       </c>
     </row>
     <row r="503">
@@ -5629,13 +5629,13 @@
     </row>
     <row r="507">
       <c r="A507" s="0">
-        <v>0.15875610617696156</v>
+        <v>0.15875610617696157</v>
       </c>
       <c r="B507" s="0">
         <v>0.022319163411138109</v>
       </c>
       <c r="C507" s="0">
-        <v>1.7738937248222117</v>
+        <v>1.7738937248222118</v>
       </c>
     </row>
     <row r="508">
@@ -5673,7 +5673,7 @@
     </row>
     <row r="511">
       <c r="A511" s="0">
-        <v>0.16001109515859765</v>
+        <v>0.16001109515859766</v>
       </c>
       <c r="B511" s="0">
         <v>0.02262045960850852</v>
@@ -5789,7 +5789,7 @@
         <v>0.023373700101934531</v>
       </c>
       <c r="C521" s="0">
-        <v>1.9454797224134281</v>
+        <v>1.9454797224134282</v>
       </c>
     </row>
     <row r="522">
@@ -5816,7 +5816,7 @@
     </row>
     <row r="524">
       <c r="A524" s="0">
-        <v>0.16408980934891484</v>
+        <v>0.16408980934891485</v>
       </c>
       <c r="B524" s="0">
         <v>0.023599672249962334</v>
@@ -5833,7 +5833,7 @@
         <v>0.023674996299304928</v>
       </c>
       <c r="C525" s="0">
-        <v>1.9959589869555538</v>
+        <v>1.9959589869555539</v>
       </c>
     </row>
     <row r="526">
@@ -5863,7 +5863,7 @@
         <v>0.16534479833055091</v>
       </c>
       <c r="B528" s="0">
-        <v>0.023900968447332738</v>
+        <v>0.023900968447332739</v>
       </c>
       <c r="C528" s="0">
         <v>2.0342427210543361</v>
@@ -5877,7 +5877,7 @@
         <v>0.023976292496675333</v>
       </c>
       <c r="C529" s="0">
-        <v>2.0470847820762494</v>
+        <v>2.0470847820762495</v>
       </c>
     </row>
     <row r="530">
@@ -5948,7 +5948,7 @@
     </row>
     <row r="536">
       <c r="A536" s="0">
-        <v>0.167854776293823</v>
+        <v>0.16785477629382301</v>
       </c>
       <c r="B536" s="0">
         <v>0.02450356084207354</v>
@@ -6039,7 +6039,7 @@
         <v>0.17036475425709513</v>
       </c>
       <c r="B544" s="0">
-        <v>0.025106153236814348</v>
+        <v>0.025106153236814349</v>
       </c>
       <c r="C544" s="0">
         <v>2.2445646767442344</v>
@@ -6185,7 +6185,7 @@
         <v>0.026085365878268162</v>
       </c>
       <c r="C557" s="0">
-        <v>2.4230682041210398</v>
+        <v>2.4230682041210399</v>
       </c>
     </row>
     <row r="558">
@@ -6196,7 +6196,7 @@
         <v>0.026160689927610763</v>
       </c>
       <c r="C558" s="0">
-        <v>2.4370821018166104</v>
+        <v>2.4370821018166105</v>
       </c>
     </row>
     <row r="559">
@@ -6369,7 +6369,7 @@
         <v>0.17977717161936557</v>
       </c>
       <c r="B574" s="0">
-        <v>0.027365874717092373</v>
+        <v>0.027365874717092374</v>
       </c>
       <c r="C574" s="0">
         <v>2.6667999748635687</v>
@@ -6380,7 +6380,7 @@
         <v>0.1800909188647746</v>
       </c>
       <c r="B575" s="0">
-        <v>0.027441198766434981</v>
+        <v>0.027441198766434982</v>
       </c>
       <c r="C575" s="0">
         <v>2.6815008112988692</v>
@@ -6391,7 +6391,7 @@
         <v>0.18040466611018363</v>
       </c>
       <c r="B576" s="0">
-        <v>0.027516522815777582</v>
+        <v>0.027516522815777583</v>
       </c>
       <c r="C576" s="0">
         <v>2.6962420558953291</v>
@@ -6460,7 +6460,7 @@
         <v>0.027968467111833182</v>
       </c>
       <c r="C582" s="0">
-        <v>2.78553809485846</v>
+        <v>2.7855380948584601</v>
       </c>
     </row>
     <row r="583">

</xml_diff>